<commit_message>
Corrige GWP biogénico CH4 (AR6), tema claro/oscuro y agrega README
- Separa el GWP de CH4 fósil (29,8) y biogénico (27,2) según IPCC AR6,
  aplicado a fermentación entérica, gestión de estiércol y efluentes
- El dashboard ahora se adapta a los 3 temas de Streamlit (oscuro/claro/sistema)
  en vez de forzar un tema único, evitando la mezcla de colores
- Reemplaza use_container_width (deprecado) por width="stretch"
- Agrega notas de verificación anual del factor CAMMESA
- Agrega README con metodología, normativa y guía de uso
- Agrega .streamlit/config.toml con tema oscuro por defecto

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Matriz_HuellaCarbono_Agropecuario.xlsx
+++ b/Matriz_HuellaCarbono_Agropecuario.xlsx
@@ -1078,7 +1078,7 @@
       </c>
       <c r="G11" s="8" t="inlineStr">
         <is>
-          <t>0,383</t>
+          <t>0,383 (CAMMESA 2023 — verificar valor vigente cada año)</t>
         </is>
       </c>
       <c r="H11" s="9" t="n"/>
@@ -1096,12 +1096,12 @@
       <c r="E12" s="6" t="n"/>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>PRG CH4 — 100 años (AR6)</t>
+          <t>PRG CH4 fósil — 100 años (AR6)</t>
         </is>
       </c>
       <c r="G12" s="8" t="inlineStr">
         <is>
-          <t>29,8</t>
+          <t>29,8 (combustión gasoil/GLP)</t>
         </is>
       </c>
       <c r="H12" s="9" t="n"/>
@@ -1119,12 +1119,12 @@
       <c r="E13" s="6" t="n"/>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>PRG N2O — 100 años (AR6)</t>
+          <t>PRG CH4 biogénico — 100 años (AR6)</t>
         </is>
       </c>
       <c r="G13" s="8" t="inlineStr">
         <is>
-          <t>273</t>
+          <t>27,2 (ganadería/efluentes)</t>
         </is>
       </c>
       <c r="H13" s="9" t="n"/>
@@ -1142,12 +1142,12 @@
       <c r="E14" s="6" t="n"/>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>Unidad de reporte</t>
+          <t>PRG N2O — 100 años (AR6)</t>
         </is>
       </c>
       <c r="G14" s="8" t="inlineStr">
         <is>
-          <t>tCO2e / año</t>
+          <t>273</t>
         </is>
       </c>
       <c r="H14" s="9" t="n"/>
@@ -1165,12 +1165,12 @@
       <c r="E15" s="6" t="n"/>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>Versión del protocolo GHG</t>
+          <t>Unidad de reporte</t>
         </is>
       </c>
       <c r="G15" s="8" t="inlineStr">
         <is>
-          <t>Corporate Standard Rev. 2015</t>
+          <t>tCO2e / año</t>
         </is>
       </c>
       <c r="H15" s="9" t="n"/>
@@ -1188,18 +1188,31 @@
       <c r="E16" s="6" t="n"/>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>Norma de referencia</t>
+          <t>Versión del protocolo GHG</t>
         </is>
       </c>
       <c r="G16" s="8" t="inlineStr">
         <is>
-          <t>ISO 14064-1:2018</t>
+          <t>Corporate Standard Rev. 2015</t>
         </is>
       </c>
       <c r="H16" s="9" t="n"/>
       <c r="I16" s="9" t="n"/>
     </row>
-    <row r="17" ht="12" customHeight="1"/>
+    <row r="17" ht="12" customHeight="1">
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t>Norma de referencia</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>ISO 14064-1:2018</t>
+        </is>
+      </c>
+      <c r="H17" s="9" t="n"/>
+      <c r="I17" s="9" t="n"/>
+    </row>
     <row r="18" ht="28" customHeight="1">
       <c r="A18" s="10" t="inlineStr">
         <is>
@@ -1407,7 +1420,7 @@
       <c r="I30" s="19" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="42">
+  <mergeCells count="43">
     <mergeCell ref="B9:E9"/>
     <mergeCell ref="G10:I10"/>
     <mergeCell ref="G6:I6"/>
@@ -1447,6 +1460,7 @@
     <mergeCell ref="C19:D19"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="G8:I8"/>
+    <mergeCell ref="G17:I17"/>
     <mergeCell ref="B10:E10"/>
     <mergeCell ref="G7:I7"/>
     <mergeCell ref="B26:I26"/>
@@ -3474,7 +3488,7 @@
     <row r="2">
       <c r="A2" s="24" t="inlineStr">
         <is>
-          <t>IPCC 2006 Vol.4 Cap.10/11  |  Tier 1 por defecto — upgradeble a Tier 2 con datos de peso y dieta  |  PRG CH4 = 29,8  |  PRG N2O = 273  (AR6, 100 años)</t>
+          <t>IPCC 2006 Vol.4 Cap.10/11  |  Tier 1 por defecto — upgradeble a Tier 2 con datos de peso y dieta  |  PRG CH4 biogénico = 27,2  |  PRG N2O = 273  (AR6, 100 años)</t>
         </is>
       </c>
     </row>
@@ -3603,7 +3617,7 @@
         <v/>
       </c>
       <c r="I6" s="28">
-        <f>H6*29.8</f>
+        <f>H6*27.2</f>
         <v/>
       </c>
       <c r="J6" s="5" t="n"/>
@@ -3644,7 +3658,7 @@
         <v/>
       </c>
       <c r="I7" s="28">
-        <f>H7*29.8</f>
+        <f>H7*27.2</f>
         <v/>
       </c>
       <c r="J7" s="5" t="n"/>
@@ -3681,7 +3695,7 @@
         <v/>
       </c>
       <c r="I8" s="28">
-        <f>H8*29.8</f>
+        <f>H8*27.2</f>
         <v/>
       </c>
       <c r="J8" s="5" t="n"/>
@@ -3718,7 +3732,7 @@
         <v/>
       </c>
       <c r="I9" s="28">
-        <f>H9*29.8</f>
+        <f>H9*27.2</f>
         <v/>
       </c>
       <c r="J9" s="5" t="n"/>
@@ -3759,7 +3773,7 @@
         <v/>
       </c>
       <c r="I10" s="28">
-        <f>H10*29.8</f>
+        <f>H10*27.2</f>
         <v/>
       </c>
       <c r="J10" s="5" t="n"/>
@@ -3800,7 +3814,7 @@
         <v/>
       </c>
       <c r="I11" s="28">
-        <f>H11*29.8</f>
+        <f>H11*27.2</f>
         <v/>
       </c>
       <c r="J11" s="5" t="n"/>
@@ -3841,7 +3855,7 @@
         <v/>
       </c>
       <c r="I12" s="28">
-        <f>H12*29.8</f>
+        <f>H12*27.2</f>
         <v/>
       </c>
       <c r="J12" s="5" t="n"/>
@@ -3882,7 +3896,7 @@
         <v/>
       </c>
       <c r="I13" s="28">
-        <f>H13*29.8</f>
+        <f>H13*27.2</f>
         <v/>
       </c>
       <c r="J13" s="5" t="n"/>
@@ -3923,7 +3937,7 @@
         <v/>
       </c>
       <c r="I14" s="28">
-        <f>H14*29.8</f>
+        <f>H14*27.2</f>
         <v/>
       </c>
       <c r="J14" s="5" t="n"/>
@@ -3964,7 +3978,7 @@
         <v/>
       </c>
       <c r="I15" s="28">
-        <f>H15*29.8</f>
+        <f>H15*27.2</f>
         <v/>
       </c>
       <c r="J15" s="5" t="n"/>
@@ -4135,7 +4149,7 @@
         <v/>
       </c>
       <c r="K20" s="28">
-        <f>I20*29.8</f>
+        <f>I20*27.2</f>
         <v/>
       </c>
       <c r="L20" s="28">
@@ -4186,7 +4200,7 @@
         <v/>
       </c>
       <c r="K21" s="28">
-        <f>I21*29.8</f>
+        <f>I21*27.2</f>
         <v/>
       </c>
       <c r="L21" s="28">
@@ -4237,7 +4251,7 @@
         <v/>
       </c>
       <c r="K22" s="28">
-        <f>I22*29.8</f>
+        <f>I22*27.2</f>
         <v/>
       </c>
       <c r="L22" s="28">
@@ -4288,7 +4302,7 @@
         <v/>
       </c>
       <c r="K23" s="28">
-        <f>I23*29.8</f>
+        <f>I23*27.2</f>
         <v/>
       </c>
       <c r="L23" s="28">
@@ -5408,7 +5422,7 @@
         <v/>
       </c>
       <c r="K5" s="28">
-        <f>J5*0.00067*1000*29.8</f>
+        <f>J5*0.00067*1000*27.2</f>
         <v/>
       </c>
       <c r="L5" s="28">
@@ -5450,7 +5464,7 @@
         <v/>
       </c>
       <c r="K6" s="28">
-        <f>J6*0.00067*1000*29.8</f>
+        <f>J6*0.00067*1000*27.2</f>
         <v/>
       </c>
       <c r="L6" s="28">
@@ -5492,7 +5506,7 @@
         <v/>
       </c>
       <c r="K7" s="28">
-        <f>J7*0.00067*1000*29.8</f>
+        <f>J7*0.00067*1000*27.2</f>
         <v/>
       </c>
       <c r="L7" s="28">
@@ -5534,7 +5548,7 @@
         <v/>
       </c>
       <c r="K8" s="28">
-        <f>J8*0.00067*1000*29.8</f>
+        <f>J8*0.00067*1000*27.2</f>
         <v/>
       </c>
       <c r="L8" s="28">
@@ -5829,7 +5843,7 @@
     <row r="2">
       <c r="A2" s="38" t="inlineStr">
         <is>
-          <t>GHG Protocol — Scope 2 Guidance (2015)  |  Factor de Emisión Red Argentina CAMMESA 2023: 0,383 kg CO2e/kWh  |  20% del consumo eléctrico total es de red; 80% autogenerado (incluido en S1-2)</t>
+          <t>GHG Protocol — Scope 2 Guidance (2015)  |  Factor de Emisión Red Argentina CAMMESA 2023: 0,383 kg CO2e/kWh (⚠ verificar valor vigente del año del inventario en cammesaweb.cammesa.com)  |  20% del consumo eléctrico total es de red; 80% autogenerado (incluido en S1-2)</t>
         </is>
       </c>
     </row>
@@ -6880,7 +6894,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H42"/>
+  <dimension ref="A1:H44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -7256,776 +7270,852 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="50" t="inlineStr">
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="35" t="inlineStr">
+        <is>
+          <t>⚠ Verificar vigencia anual</t>
+        </is>
+      </c>
+      <c r="B16" s="26" t="inlineStr">
+        <is>
+          <t>Actualizar con el valor publicado del año del inventario</t>
+        </is>
+      </c>
+      <c r="C16" s="26" t="inlineStr">
+        <is>
+          <t>kWh</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G16" s="52" t="inlineStr">
+        <is>
+          <t>cammesaweb.cammesa.com/download/factor-de-emision</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="50" t="inlineStr">
         <is>
           <t>GANADERÍA — FERMENTACIÓN ENTÉRICA (Tier 1, clima templado)</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="51" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="51" t="inlineStr">
         <is>
           <t>Gas / Fuente</t>
         </is>
       </c>
-      <c r="B18" s="51" t="inlineStr">
+      <c r="B19" s="51" t="inlineStr">
         <is>
           <t>Aplicación</t>
         </is>
       </c>
-      <c r="C18" s="51" t="inlineStr">
+      <c r="C19" s="51" t="inlineStr">
         <is>
           <t>Unidad</t>
         </is>
       </c>
-      <c r="D18" s="51" t="inlineStr">
+      <c r="D19" s="51" t="inlineStr">
         <is>
           <t>FE CO2 (kg CO2/unidad)</t>
         </is>
       </c>
-      <c r="E18" s="51" t="inlineStr">
+      <c r="E19" s="51" t="inlineStr">
         <is>
           <t>FE CH4 (g/unidad)</t>
         </is>
       </c>
-      <c r="F18" s="51" t="inlineStr">
+      <c r="F19" s="51" t="inlineStr">
         <is>
           <t>FE N2O (g/unidad)</t>
         </is>
       </c>
-      <c r="G18" s="51" t="inlineStr">
+      <c r="G19" s="51" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="H18" s="19" t="n"/>
-    </row>
-    <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="35" t="inlineStr">
+      <c r="H19" s="19" t="n"/>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="35" t="inlineStr">
         <is>
           <t>Vacas lecheras (&gt;200 L/día producción)</t>
         </is>
       </c>
-      <c r="B19" s="26" t="inlineStr">
+      <c r="B20" s="26" t="inlineStr">
         <is>
           <t>Fermentación entérica</t>
         </is>
       </c>
-      <c r="C19" s="26" t="inlineStr">
+      <c r="C20" s="26" t="inlineStr">
         <is>
           <t>cab/año</t>
         </is>
       </c>
-      <c r="D19" s="8" t="inlineStr">
+      <c r="D20" s="8" t="inlineStr">
         <is>
           <t>119,8 kg CH4</t>
         </is>
       </c>
-      <c r="E19" s="8" t="inlineStr">
+      <c r="E20" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F19" s="8" t="inlineStr">
+      <c r="F20" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G19" s="52" t="inlineStr">
+      <c r="G20" s="52" t="inlineStr">
         <is>
           <t>IPCC 2006 Tabla 10-11</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="36" t="inlineStr">
+    <row r="21" ht="18" customHeight="1">
+      <c r="A21" s="36" t="inlineStr">
         <is>
           <t>Bovinos adultos carne (&gt;300 kg)</t>
         </is>
       </c>
-      <c r="B20" s="29" t="inlineStr">
+      <c r="B21" s="29" t="inlineStr">
         <is>
           <t>Fermentación entérica</t>
         </is>
       </c>
-      <c r="C20" s="29" t="inlineStr">
+      <c r="C21" s="29" t="inlineStr">
         <is>
           <t>cab/año</t>
         </is>
       </c>
-      <c r="D20" s="8" t="inlineStr">
+      <c r="D21" s="8" t="inlineStr">
         <is>
           <t>56,5 kg CH4</t>
         </is>
       </c>
-      <c r="E20" s="8" t="inlineStr">
+      <c r="E21" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F20" s="8" t="inlineStr">
+      <c r="F21" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G20" s="52" t="inlineStr">
+      <c r="G21" s="52" t="inlineStr">
         <is>
           <t>IPCC 2006 Tabla 10-11</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="35" t="inlineStr">
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="35" t="inlineStr">
         <is>
           <t>Novillo / vaquillona recría (200-300 kg)</t>
         </is>
       </c>
-      <c r="B21" s="26" t="inlineStr">
+      <c r="B22" s="26" t="inlineStr">
         <is>
           <t>Fermentación entérica</t>
         </is>
       </c>
-      <c r="C21" s="26" t="inlineStr">
+      <c r="C22" s="26" t="inlineStr">
         <is>
           <t>cab/año</t>
         </is>
       </c>
-      <c r="D21" s="8" t="inlineStr">
+      <c r="D22" s="8" t="inlineStr">
         <is>
           <t>47,8 kg CH4</t>
         </is>
       </c>
-      <c r="E21" s="8" t="inlineStr">
+      <c r="E22" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F21" s="8" t="inlineStr">
+      <c r="F22" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G21" s="52" t="inlineStr">
+      <c r="G22" s="52" t="inlineStr">
         <is>
           <t>IPCC 2006 Tabla 10-11</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="36" t="inlineStr">
+    <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="36" t="inlineStr">
         <is>
           <t>Terneros &lt; 1 año</t>
         </is>
       </c>
-      <c r="B22" s="29" t="inlineStr">
+      <c r="B23" s="29" t="inlineStr">
         <is>
           <t>Fermentación entérica</t>
         </is>
       </c>
-      <c r="C22" s="29" t="inlineStr">
+      <c r="C23" s="29" t="inlineStr">
         <is>
           <t>cab/año</t>
         </is>
       </c>
-      <c r="D22" s="8" t="inlineStr">
+      <c r="D23" s="8" t="inlineStr">
         <is>
           <t>27,0 kg CH4</t>
         </is>
       </c>
-      <c r="E22" s="8" t="inlineStr">
+      <c r="E23" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F22" s="8" t="inlineStr">
+      <c r="F23" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G22" s="52" t="inlineStr">
+      <c r="G23" s="52" t="inlineStr">
         <is>
           <t>IPCC 2006 Tabla 10-11</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="35" t="inlineStr">
+    <row r="24" ht="18" customHeight="1">
+      <c r="A24" s="35" t="inlineStr">
         <is>
           <t>Toros reproductores</t>
         </is>
       </c>
-      <c r="B23" s="26" t="inlineStr">
+      <c r="B24" s="26" t="inlineStr">
         <is>
           <t>Fermentación entérica</t>
         </is>
       </c>
-      <c r="C23" s="26" t="inlineStr">
+      <c r="C24" s="26" t="inlineStr">
         <is>
           <t>cab/año</t>
         </is>
       </c>
-      <c r="D23" s="8" t="inlineStr">
+      <c r="D24" s="8" t="inlineStr">
         <is>
           <t>73,0 kg CH4</t>
         </is>
       </c>
-      <c r="E23" s="8" t="inlineStr">
+      <c r="E24" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F23" s="8" t="inlineStr">
+      <c r="F24" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G23" s="52" t="inlineStr">
+      <c r="G24" s="52" t="inlineStr">
         <is>
           <t>IPCC 2006 Tabla 10-11</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="36" t="inlineStr">
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="36" t="inlineStr">
         <is>
           <t>Ovinos (adultos)</t>
         </is>
       </c>
-      <c r="B24" s="29" t="inlineStr">
+      <c r="B25" s="29" t="inlineStr">
         <is>
           <t>Fermentación entérica</t>
         </is>
       </c>
-      <c r="C24" s="29" t="inlineStr">
+      <c r="C25" s="29" t="inlineStr">
         <is>
           <t>cab/año</t>
         </is>
       </c>
-      <c r="D24" s="8" t="inlineStr">
+      <c r="D25" s="8" t="inlineStr">
         <is>
           <t>8,0 kg CH4</t>
         </is>
       </c>
-      <c r="E24" s="8" t="inlineStr">
+      <c r="E25" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F24" s="8" t="inlineStr">
+      <c r="F25" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G24" s="52" t="inlineStr">
+      <c r="G25" s="52" t="inlineStr">
         <is>
           <t>IPCC 2006 Tabla 10-11</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="22" customHeight="1">
-      <c r="A26" s="50" t="inlineStr">
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="50" t="inlineStr">
         <is>
           <t>GANADERÍA — GESTIÓN DE ESTIÉRCOL (Tier 1)</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="51" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="51" t="inlineStr">
         <is>
           <t>Gas / Fuente</t>
         </is>
       </c>
-      <c r="B27" s="51" t="inlineStr">
+      <c r="B28" s="51" t="inlineStr">
         <is>
           <t>Aplicación</t>
         </is>
       </c>
-      <c r="C27" s="51" t="inlineStr">
+      <c r="C28" s="51" t="inlineStr">
         <is>
           <t>Unidad</t>
         </is>
       </c>
-      <c r="D27" s="51" t="inlineStr">
+      <c r="D28" s="51" t="inlineStr">
         <is>
           <t>FE CO2 (kg CO2/unidad)</t>
         </is>
       </c>
-      <c r="E27" s="51" t="inlineStr">
+      <c r="E28" s="51" t="inlineStr">
         <is>
           <t>FE CH4 (g/unidad)</t>
         </is>
       </c>
-      <c r="F27" s="51" t="inlineStr">
+      <c r="F28" s="51" t="inlineStr">
         <is>
           <t>FE N2O (g/unidad)</t>
         </is>
       </c>
-      <c r="G27" s="51" t="inlineStr">
+      <c r="G28" s="51" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="H27" s="19" t="n"/>
-    </row>
-    <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="35" t="inlineStr">
+      <c r="H28" s="19" t="n"/>
+    </row>
+    <row r="29" ht="18" customHeight="1">
+      <c r="A29" s="35" t="inlineStr">
         <is>
           <t>Vacas lecheras — laguna anaeróbica</t>
         </is>
       </c>
-      <c r="B28" s="26" t="inlineStr">
+      <c r="B29" s="26" t="inlineStr">
         <is>
           <t>CH4 estiércol</t>
         </is>
       </c>
-      <c r="C28" s="26" t="inlineStr">
+      <c r="C29" s="26" t="inlineStr">
         <is>
           <t>cab/año</t>
         </is>
       </c>
-      <c r="D28" s="8" t="inlineStr">
+      <c r="D29" s="8" t="inlineStr">
         <is>
           <t>16,0 kg CH4</t>
         </is>
       </c>
-      <c r="E28" s="8" t="inlineStr">
+      <c r="E29" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F28" s="8" t="inlineStr">
+      <c r="F29" s="8" t="inlineStr">
         <is>
           <t>0,10 kg N2O</t>
         </is>
       </c>
-      <c r="G28" s="52" t="inlineStr">
+      <c r="G29" s="52" t="inlineStr">
         <is>
           <t>IPCC 2006 Tabla 10-14/15</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="36" t="inlineStr">
+    <row r="30" ht="18" customHeight="1">
+      <c r="A30" s="36" t="inlineStr">
         <is>
           <t>Bovinos carne — almac. sólido/corral</t>
         </is>
       </c>
-      <c r="B29" s="29" t="inlineStr">
+      <c r="B30" s="29" t="inlineStr">
         <is>
           <t>CH4 estiércol</t>
         </is>
       </c>
-      <c r="C29" s="29" t="inlineStr">
+      <c r="C30" s="29" t="inlineStr">
         <is>
           <t>cab/año</t>
         </is>
       </c>
-      <c r="D29" s="8" t="inlineStr">
+      <c r="D30" s="8" t="inlineStr">
         <is>
           <t>1,0 kg CH4</t>
         </is>
       </c>
-      <c r="E29" s="8" t="inlineStr">
+      <c r="E30" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F29" s="8" t="inlineStr">
+      <c r="F30" s="8" t="inlineStr">
         <is>
           <t>0,20 kg N2O</t>
         </is>
       </c>
-      <c r="G29" s="52" t="inlineStr">
+      <c r="G30" s="52" t="inlineStr">
         <is>
           <t>IPCC 2006 Tabla 10-14/15</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="35" t="inlineStr">
+    <row r="31" ht="18" customHeight="1">
+      <c r="A31" s="35" t="inlineStr">
         <is>
           <t>Bovinos — pastoreo directo</t>
         </is>
       </c>
-      <c r="B30" s="26" t="inlineStr">
+      <c r="B31" s="26" t="inlineStr">
         <is>
           <t>CH4 estiércol</t>
         </is>
       </c>
-      <c r="C30" s="26" t="inlineStr">
+      <c r="C31" s="26" t="inlineStr">
         <is>
           <t>cab/año</t>
         </is>
       </c>
-      <c r="D30" s="8" t="inlineStr">
+      <c r="D31" s="8" t="inlineStr">
         <is>
           <t>1,0 kg CH4</t>
         </is>
       </c>
-      <c r="E30" s="8" t="inlineStr">
+      <c r="E31" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F30" s="8" t="inlineStr">
+      <c r="F31" s="8" t="inlineStr">
         <is>
           <t>0,07 kg N2O</t>
         </is>
       </c>
-      <c r="G30" s="52" t="inlineStr">
+      <c r="G31" s="52" t="inlineStr">
         <is>
           <t>IPCC 2006 Tabla 10-14/15</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="22" customHeight="1">
-      <c r="A32" s="50" t="inlineStr">
+    <row r="33" ht="22" customHeight="1">
+      <c r="A33" s="50" t="inlineStr">
         <is>
           <t>SUELOS AGRÍCOLAS</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="51" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="51" t="inlineStr">
         <is>
           <t>Gas / Fuente</t>
         </is>
       </c>
-      <c r="B33" s="51" t="inlineStr">
+      <c r="B34" s="51" t="inlineStr">
         <is>
           <t>Aplicación</t>
         </is>
       </c>
-      <c r="C33" s="51" t="inlineStr">
+      <c r="C34" s="51" t="inlineStr">
         <is>
           <t>Unidad</t>
         </is>
       </c>
-      <c r="D33" s="51" t="inlineStr">
+      <c r="D34" s="51" t="inlineStr">
         <is>
           <t>FE CO2 (kg CO2/unidad)</t>
         </is>
       </c>
-      <c r="E33" s="51" t="inlineStr">
+      <c r="E34" s="51" t="inlineStr">
         <is>
           <t>FE CH4 (g/unidad)</t>
         </is>
       </c>
-      <c r="F33" s="51" t="inlineStr">
+      <c r="F34" s="51" t="inlineStr">
         <is>
           <t>FE N2O (g/unidad)</t>
         </is>
       </c>
-      <c r="G33" s="51" t="inlineStr">
+      <c r="G34" s="51" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="H33" s="19" t="n"/>
-    </row>
-    <row r="34" ht="18" customHeight="1">
-      <c r="A34" s="35" t="inlineStr">
+      <c r="H34" s="19" t="n"/>
+    </row>
+    <row r="35" ht="18" customHeight="1">
+      <c r="A35" s="35" t="inlineStr">
         <is>
           <t>Fertilizante N (nitrogenado)</t>
         </is>
       </c>
-      <c r="B34" s="26" t="inlineStr">
+      <c r="B35" s="26" t="inlineStr">
         <is>
           <t>N2O directo suelos EF1</t>
         </is>
       </c>
-      <c r="C34" s="26" t="inlineStr">
+      <c r="C35" s="26" t="inlineStr">
         <is>
           <t>kg N aplic.</t>
         </is>
       </c>
-      <c r="D34" s="8" t="inlineStr">
+      <c r="D35" s="8" t="inlineStr">
         <is>
           <t>0,01 kg N2O-N</t>
         </is>
       </c>
-      <c r="E34" s="8" t="inlineStr">
+      <c r="E35" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F34" s="8" t="inlineStr">
+      <c r="F35" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G34" s="52" t="inlineStr">
+      <c r="G35" s="52" t="inlineStr">
         <is>
           <t>IPCC 2006 Tabla 11-1</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="18" customHeight="1">
-      <c r="A35" s="36" t="inlineStr">
+    <row r="36" ht="18" customHeight="1">
+      <c r="A36" s="36" t="inlineStr">
         <is>
           <t>Urea aplicada</t>
         </is>
       </c>
-      <c r="B35" s="29" t="inlineStr">
+      <c r="B36" s="29" t="inlineStr">
         <is>
           <t>CO2 hidrólisis</t>
         </is>
       </c>
-      <c r="C35" s="29" t="inlineStr">
+      <c r="C36" s="29" t="inlineStr">
         <is>
           <t>kg urea</t>
         </is>
       </c>
-      <c r="D35" s="8" t="inlineStr">
+      <c r="D36" s="8" t="inlineStr">
         <is>
           <t>0,734 kg CO2</t>
         </is>
       </c>
-      <c r="E35" s="8" t="inlineStr">
+      <c r="E36" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F35" s="8" t="inlineStr">
+      <c r="F36" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G35" s="52" t="inlineStr">
+      <c r="G36" s="52" t="inlineStr">
         <is>
           <t>IPCC 2006 Vol.4 Cap.11</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="35" t="inlineStr">
+    <row r="37" ht="18" customHeight="1">
+      <c r="A37" s="35" t="inlineStr">
         <is>
           <t>Residuos de cultivos incorporados</t>
         </is>
       </c>
-      <c r="B36" s="26" t="inlineStr">
+      <c r="B37" s="26" t="inlineStr">
         <is>
           <t>N2O indirecto</t>
         </is>
       </c>
-      <c r="C36" s="26" t="inlineStr">
+      <c r="C37" s="26" t="inlineStr">
         <is>
           <t>kg N residuos</t>
         </is>
       </c>
-      <c r="D36" s="8" t="inlineStr">
+      <c r="D37" s="8" t="inlineStr">
         <is>
           <t>0,01 kg N2O-N</t>
         </is>
       </c>
-      <c r="E36" s="8" t="inlineStr">
+      <c r="E37" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F36" s="8" t="inlineStr">
+      <c r="F37" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G36" s="52" t="inlineStr">
+      <c r="G37" s="52" t="inlineStr">
         <is>
           <t>IPCC 2006 Tabla 11-1</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="22" customHeight="1">
-      <c r="A38" s="50" t="inlineStr">
+    <row r="39" ht="22" customHeight="1">
+      <c r="A39" s="50" t="inlineStr">
         <is>
           <t>POTENCIALES DE CALENTAMIENTO GLOBAL (AR6 — 100 años)</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="51" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="51" t="inlineStr">
         <is>
           <t>Gas / Fuente</t>
         </is>
       </c>
-      <c r="B39" s="51" t="inlineStr">
+      <c r="B40" s="51" t="inlineStr">
         <is>
           <t>Aplicación</t>
         </is>
       </c>
-      <c r="C39" s="51" t="inlineStr">
+      <c r="C40" s="51" t="inlineStr">
         <is>
           <t>Unidad</t>
         </is>
       </c>
-      <c r="D39" s="51" t="inlineStr">
+      <c r="D40" s="51" t="inlineStr">
         <is>
           <t>FE CO2 (kg CO2/unidad)</t>
         </is>
       </c>
-      <c r="E39" s="51" t="inlineStr">
+      <c r="E40" s="51" t="inlineStr">
         <is>
           <t>FE CH4 (g/unidad)</t>
         </is>
       </c>
-      <c r="F39" s="51" t="inlineStr">
+      <c r="F40" s="51" t="inlineStr">
         <is>
           <t>FE N2O (g/unidad)</t>
         </is>
       </c>
-      <c r="G39" s="51" t="inlineStr">
+      <c r="G40" s="51" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="H39" s="19" t="n"/>
-    </row>
-    <row r="40" ht="18" customHeight="1">
-      <c r="A40" s="35" t="inlineStr">
-        <is>
-          <t>CH4 (metano)</t>
-        </is>
-      </c>
-      <c r="B40" s="26" t="inlineStr">
+      <c r="H40" s="19" t="n"/>
+    </row>
+    <row r="41" ht="18" customHeight="1">
+      <c r="A41" s="35" t="inlineStr">
+        <is>
+          <t>CH4 fósil (combustión gasoil/GLP)</t>
+        </is>
+      </c>
+      <c r="B41" s="26" t="inlineStr">
+        <is>
+          <t>GWP base CO2 — Hojas S1-1 y S1-2</t>
+        </is>
+      </c>
+      <c r="C41" s="26" t="inlineStr">
+        <is>
+          <t>kg CH4</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>29,8 kg CO2e</t>
+        </is>
+      </c>
+      <c r="E41" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F41" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G41" s="52" t="inlineStr">
+        <is>
+          <t>IPCC AR6 2021 Tabla 7.SM.7</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="18" customHeight="1">
+      <c r="A42" s="36" t="inlineStr">
+        <is>
+          <t>CH4 biogénico (ganadería/efluentes)</t>
+        </is>
+      </c>
+      <c r="B42" s="29" t="inlineStr">
+        <is>
+          <t>GWP base CO2 — Hojas S1-3 y S1-5</t>
+        </is>
+      </c>
+      <c r="C42" s="29" t="inlineStr">
+        <is>
+          <t>kg CH4</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>27,2 kg CO2e</t>
+        </is>
+      </c>
+      <c r="E42" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F42" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G42" s="52" t="inlineStr">
+        <is>
+          <t>IPCC AR6 2021 Tabla 7.SM.7</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="18" customHeight="1">
+      <c r="A43" s="35" t="inlineStr">
+        <is>
+          <t>N2O (óxido nitroso)</t>
+        </is>
+      </c>
+      <c r="B43" s="26" t="inlineStr">
         <is>
           <t>GWP base CO2</t>
         </is>
       </c>
-      <c r="C40" s="26" t="inlineStr">
-        <is>
-          <t>kg CH4</t>
-        </is>
-      </c>
-      <c r="D40" s="8" t="inlineStr">
-        <is>
-          <t>29,8 kg CO2e</t>
-        </is>
-      </c>
-      <c r="E40" s="8" t="inlineStr">
+      <c r="C43" s="26" t="inlineStr">
+        <is>
+          <t>kg N2O</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>273 kg CO2e</t>
+        </is>
+      </c>
+      <c r="E43" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F40" s="8" t="inlineStr">
+      <c r="F43" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G40" s="52" t="inlineStr">
+      <c r="G43" s="52" t="inlineStr">
         <is>
           <t>IPCC AR6 2021 Tabla 7.SM.7</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="18" customHeight="1">
-      <c r="A41" s="36" t="inlineStr">
-        <is>
-          <t>N2O (óxido nitroso)</t>
-        </is>
-      </c>
-      <c r="B41" s="29" t="inlineStr">
+    <row r="44" ht="18" customHeight="1">
+      <c r="A44" s="36" t="inlineStr">
+        <is>
+          <t>CO2 (dióxido de carbono)</t>
+        </is>
+      </c>
+      <c r="B44" s="29" t="inlineStr">
         <is>
           <t>GWP base CO2</t>
         </is>
       </c>
-      <c r="C41" s="29" t="inlineStr">
-        <is>
-          <t>kg N2O</t>
-        </is>
-      </c>
-      <c r="D41" s="8" t="inlineStr">
-        <is>
-          <t>273 kg CO2e</t>
-        </is>
-      </c>
-      <c r="E41" s="8" t="inlineStr">
+      <c r="C44" s="29" t="inlineStr">
+        <is>
+          <t>kg CO2</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="inlineStr">
+        <is>
+          <t>1 kg CO2e</t>
+        </is>
+      </c>
+      <c r="E44" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F41" s="8" t="inlineStr">
+      <c r="F44" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G41" s="52" t="inlineStr">
-        <is>
-          <t>IPCC AR6 2021 Tabla 7.SM.7</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="18" customHeight="1">
-      <c r="A42" s="35" t="inlineStr">
-        <is>
-          <t>CO2 (dióxido de carbono)</t>
-        </is>
-      </c>
-      <c r="B42" s="26" t="inlineStr">
-        <is>
-          <t>GWP base CO2</t>
-        </is>
-      </c>
-      <c r="C42" s="26" t="inlineStr">
-        <is>
-          <t>kg CO2</t>
-        </is>
-      </c>
-      <c r="D42" s="8" t="inlineStr">
-        <is>
-          <t>1 kg CO2e</t>
-        </is>
-      </c>
-      <c r="E42" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F42" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G42" s="52" t="inlineStr">
+      <c r="G44" s="52" t="inlineStr">
         <is>
           <t>Línea base</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="36">
+  <mergeCells count="38">
     <mergeCell ref="G21:H21"/>
+    <mergeCell ref="G43:H43"/>
+    <mergeCell ref="A39:H39"/>
     <mergeCell ref="G42:H42"/>
-    <mergeCell ref="G27:H27"/>
     <mergeCell ref="G36:H36"/>
     <mergeCell ref="G23:H23"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="G8:H8"/>
-    <mergeCell ref="G39:H39"/>
     <mergeCell ref="G7:H7"/>
     <mergeCell ref="G10:H10"/>
     <mergeCell ref="G19:H19"/>
+    <mergeCell ref="G37:H37"/>
     <mergeCell ref="G28:H28"/>
     <mergeCell ref="G6:H6"/>
     <mergeCell ref="G13:H13"/>
-    <mergeCell ref="G18:H18"/>
+    <mergeCell ref="A27:H27"/>
     <mergeCell ref="A12:H12"/>
-    <mergeCell ref="A26:H26"/>
+    <mergeCell ref="A18:H18"/>
     <mergeCell ref="G34:H34"/>
     <mergeCell ref="G24:H24"/>
     <mergeCell ref="G30:H30"/>
     <mergeCell ref="G15:H15"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="G33:H33"/>
     <mergeCell ref="G5:H5"/>
+    <mergeCell ref="A33:H33"/>
     <mergeCell ref="G14:H14"/>
-    <mergeCell ref="A32:H32"/>
-    <mergeCell ref="A17:H17"/>
     <mergeCell ref="G29:H29"/>
     <mergeCell ref="A4:H4"/>
     <mergeCell ref="G35:H35"/>
     <mergeCell ref="G20:H20"/>
-    <mergeCell ref="A38:H38"/>
+    <mergeCell ref="G16:H16"/>
+    <mergeCell ref="G25:H25"/>
     <mergeCell ref="G41:H41"/>
+    <mergeCell ref="G31:H31"/>
+    <mergeCell ref="G44:H44"/>
     <mergeCell ref="G22:H22"/>
     <mergeCell ref="G40:H40"/>
     <mergeCell ref="G9:H9"/>

</xml_diff>